<commit_message>
adjusted test data to use accurate fields
</commit_message>
<xml_diff>
--- a/rules/CORE-001080/negative/02/data/unit-test-coreid-CG0288-negative 2.xlsx
+++ b/rules/CORE-001080/negative/02/data/unit-test-coreid-CG0288-negative 2.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -58,8 +58,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -67,6 +71,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -96,13 +106,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,10 +465,10 @@
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" s="4" t="str">
-        <v>sdtmct-2026-03-27</v>
+        <v>sdtmct</v>
       </c>
       <c r="B3" s="4" t="str" xml:space="preserve">
-        <v xml:space="preserve">
+        <v xml:space="preserve">2024-09-27
 </v>
       </c>
     </row>
@@ -798,13 +809,13 @@
       <c r="H6" s="4" t="str">
         <v/>
       </c>
-      <c r="I6" s="5" t="str">
+      <c r="I6" s="6" t="str">
         <v>C128949</v>
       </c>
-      <c r="J6" s="5" t="str">
+      <c r="J6" s="6" t="str">
         <v>CDISC CT</v>
       </c>
-      <c r="K6" s="5" t="str">
+      <c r="K6" s="6" t="str">
         <v>2016-06-24</v>
       </c>
     </row>

</xml_diff>